<commit_message>
Release v1.2.1: improve promoter transaction analysis
</commit_message>
<xml_diff>
--- a/output/2026-08-17/enriched_analysis.xlsx
+++ b/output/2026-08-17/enriched_analysis.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ScoredStocks" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="FilteredStocks" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ScoredStocks" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FilteredStocks" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,16 +19,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +36,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -47,21 +44,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -427,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC39"/>
+  <dimension ref="A1:AC40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -462,147 +450,147 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Symbol</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>CompanyName</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>ScorePromo</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>ScoreFund</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>ScoreTech</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>ScoreRisk</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>LastPrice</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>AvgPrice</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>PriceDiffPct</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>PromoHolding</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>ValueCr</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>NumBuyTxn</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>acqtoDt</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>PromoConvictionPct</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>MarketCapCr</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>PE</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>RevGrowthPct</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>EBITDAGrowthPct</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>PATGrowthPct</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>EPSGrowthPct</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>ROCEPct</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>DE_Ratio</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>OCFPositive</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>OPMPct</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>DMA50</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>DMA200</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>SixMonthReturn</t>
         </is>
@@ -663,13 +651,13 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>0.082</v>
+        <v>0.08</v>
       </c>
       <c r="Q2" t="n">
-        <v>2419</v>
+        <v>2493</v>
       </c>
       <c r="R2" t="n">
-        <v>8.31</v>
+        <v>8.57</v>
       </c>
       <c r="S2" t="n">
         <v>36</v>
@@ -708,16 +696,16 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MACPOWER</t>
+          <t>PREMIERPOL</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MACPOWER CNC MACHINES LIMITED</t>
+          <t>PREMIER POLYFILM LIMITED</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -725,10 +713,10 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="F3" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G3" t="n">
         <v>30</v>
@@ -737,84 +725,84 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>1798</v>
+        <v>85.45</v>
       </c>
       <c r="J3" t="n">
-        <v>920.51</v>
+        <v>54.77</v>
       </c>
       <c r="K3" t="n">
-        <v>95.3</v>
+        <v>56</v>
       </c>
       <c r="L3" t="n">
-        <v>73.16</v>
+        <v>67.45999999999999</v>
       </c>
       <c r="M3" t="n">
-        <v>0.44</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="N3" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>04-06-2026</t>
+          <t>17-06-2026</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>0.025</v>
+        <v>0.926</v>
       </c>
       <c r="Q3" t="n">
-        <v>1782</v>
+        <v>905</v>
       </c>
       <c r="R3" t="n">
-        <v>45.8</v>
+        <v>25.9</v>
       </c>
       <c r="S3" t="n">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="T3" t="n">
-        <v>15.42</v>
+        <v>13.52</v>
       </c>
       <c r="U3" t="n">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="V3" t="n">
-        <v>9.58</v>
+        <v>0.87</v>
       </c>
       <c r="W3" t="n">
-        <v>29.1</v>
+        <v>30.8</v>
       </c>
       <c r="X3" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="Y3" t="b">
         <v>1</v>
       </c>
       <c r="Z3" t="n">
-        <v>16.19</v>
+        <v>15.38</v>
       </c>
       <c r="AA3" t="n">
-        <v>1345.02</v>
+        <v>67.64</v>
       </c>
       <c r="AB3" t="n">
-        <v>1060.64</v>
+        <v>54.56</v>
       </c>
       <c r="AC3" t="n">
-        <v>97.2</v>
+        <v>56.4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>APLLTD</t>
+          <t>MACPOWER</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Alembic Pharmaceuticals Limited</t>
+          <t>MACPOWER CNC MACHINES LIMITED</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -822,10 +810,10 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F4" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G4" t="n">
         <v>30</v>
@@ -834,84 +822,84 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>823.8</v>
+        <v>1798</v>
       </c>
       <c r="J4" t="n">
-        <v>754.37</v>
+        <v>920.51</v>
       </c>
       <c r="K4" t="n">
-        <v>9.199999999999999</v>
+        <v>95.3</v>
       </c>
       <c r="L4" t="n">
-        <v>69.61</v>
+        <v>73.16</v>
       </c>
       <c r="M4" t="n">
-        <v>24.22</v>
+        <v>0.44</v>
       </c>
       <c r="N4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>04-06-2026</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>0.15</v>
+        <v>0.022</v>
       </c>
       <c r="Q4" t="n">
-        <v>16167</v>
+        <v>1984</v>
       </c>
       <c r="R4" t="n">
-        <v>20.5</v>
+        <v>51</v>
       </c>
       <c r="S4" t="n">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="T4" t="n">
-        <v>346</v>
+        <v>15.42</v>
       </c>
       <c r="U4" t="n">
-        <v>88</v>
+        <v>47</v>
       </c>
       <c r="V4" t="n">
-        <v>10.02</v>
+        <v>9.58</v>
       </c>
       <c r="W4" t="n">
-        <v>12.3</v>
+        <v>29.1</v>
       </c>
       <c r="X4" t="n">
-        <v>0.21</v>
+        <v>0.01</v>
       </c>
       <c r="Y4" t="b">
         <v>1</v>
       </c>
       <c r="Z4" t="n">
-        <v>19</v>
+        <v>16.19</v>
       </c>
       <c r="AA4" t="n">
-        <v>802.9299999999999</v>
+        <v>1345.02</v>
       </c>
       <c r="AB4" t="n">
-        <v>796.76</v>
+        <v>1060.64</v>
       </c>
       <c r="AC4" t="n">
-        <v>2.6</v>
+        <v>97.2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>THANGAMAYL</t>
+          <t>APLLTD</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>THANGAMAYIL JEWELLERY LIMITED</t>
+          <t>Alembic Pharmaceuticals Limited</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -922,93 +910,93 @@
         <v>20</v>
       </c>
       <c r="F5" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="G5" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>5329</v>
+        <v>823.8</v>
       </c>
       <c r="J5" t="n">
-        <v>5085.36</v>
+        <v>753.55</v>
       </c>
       <c r="K5" t="n">
-        <v>4.8</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="L5" t="n">
-        <v>67.16</v>
+        <v>69.61</v>
       </c>
       <c r="M5" t="n">
-        <v>5.22</v>
+        <v>19.68</v>
       </c>
       <c r="N5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>07-08-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>0.031</v>
+        <v>0.121</v>
       </c>
       <c r="Q5" t="n">
-        <v>16583</v>
+        <v>16199</v>
       </c>
       <c r="R5" t="n">
-        <v>42.2</v>
+        <v>20.5</v>
       </c>
       <c r="S5" t="n">
-        <v>83</v>
+        <v>16</v>
       </c>
       <c r="T5" t="n">
-        <v>145</v>
+        <v>346</v>
       </c>
       <c r="U5" t="n">
-        <v>264</v>
+        <v>88</v>
       </c>
       <c r="V5" t="n">
-        <v>27.38</v>
+        <v>10.02</v>
       </c>
       <c r="W5" t="n">
-        <v>25.5</v>
+        <v>12.3</v>
       </c>
       <c r="X5" t="n">
-        <v>0.64</v>
+        <v>0.21</v>
       </c>
       <c r="Y5" t="b">
         <v>1</v>
       </c>
       <c r="Z5" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="AA5" t="n">
-        <v>5884.22</v>
+        <v>802.9299999999999</v>
       </c>
       <c r="AB5" t="n">
-        <v>4134.2</v>
+        <v>796.76</v>
       </c>
       <c r="AC5" t="n">
-        <v>44.1</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CHEMBONDCH</t>
+          <t>THANGAMAYL</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CHEMBOND CHEMICALS LIMITED</t>
+          <t>THANGAMAYIL JEWELLERY LIMITED</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1019,78 +1007,78 @@
         <v>20</v>
       </c>
       <c r="F6" t="n">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G6" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>264</v>
+        <v>5329</v>
       </c>
       <c r="J6" t="n">
-        <v>230</v>
+        <v>5085.36</v>
       </c>
       <c r="K6" t="n">
-        <v>14.8</v>
+        <v>4.8</v>
       </c>
       <c r="L6" t="n">
-        <v>67.65000000000001</v>
+        <v>67.16</v>
       </c>
       <c r="M6" t="n">
-        <v>1.4</v>
+        <v>5.22</v>
       </c>
       <c r="N6" t="n">
         <v>4</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>06-08-2026</t>
+          <t>07-08-2026</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>0.198</v>
+        <v>0.031</v>
       </c>
       <c r="Q6" t="n">
-        <v>706</v>
+        <v>17046</v>
       </c>
       <c r="R6" t="n">
-        <v>59</v>
+        <v>43.4</v>
       </c>
       <c r="S6" t="n">
-        <v>3</v>
+        <v>83</v>
       </c>
       <c r="T6" t="n">
-        <v>2.99</v>
+        <v>145</v>
       </c>
       <c r="U6" t="n">
-        <v>97</v>
+        <v>264</v>
       </c>
       <c r="V6" t="n">
-        <v>1</v>
+        <v>27.38</v>
       </c>
       <c r="W6" t="n">
-        <v>11.6</v>
+        <v>25.5</v>
       </c>
       <c r="X6" t="n">
-        <v>0</v>
+        <v>0.64</v>
       </c>
       <c r="Y6" t="b">
         <v>1</v>
       </c>
       <c r="Z6" t="n">
-        <v>16.21</v>
+        <v>5</v>
       </c>
       <c r="AA6" t="n">
-        <v>228.71</v>
+        <v>5884.22</v>
       </c>
       <c r="AB6" t="n">
-        <v>172.77</v>
+        <v>4134.2</v>
       </c>
       <c r="AC6" t="n">
-        <v>66.3</v>
+        <v>44.1</v>
       </c>
     </row>
     <row r="7">
@@ -1128,10 +1116,10 @@
         <v>576</v>
       </c>
       <c r="J7" t="n">
-        <v>374.61</v>
+        <v>379.74</v>
       </c>
       <c r="K7" t="n">
-        <v>53.8</v>
+        <v>51.7</v>
       </c>
       <c r="L7" t="n">
         <v>63.09</v>
@@ -1140,7 +1128,7 @@
         <v>13.87</v>
       </c>
       <c r="N7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1148,13 +1136,13 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>0.76</v>
+        <v>0.763</v>
       </c>
       <c r="Q7" t="n">
-        <v>1824</v>
+        <v>1817</v>
       </c>
       <c r="R7" t="n">
-        <v>21.6</v>
+        <v>21.5</v>
       </c>
       <c r="S7" t="n">
         <v>581</v>
@@ -1191,12 +1179,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>STEL</t>
+          <t>EUROPRATIK</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>STEL HOLDINGS LIMITED</t>
+          <t>Euro Pratik Sales Limited</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1208,81 +1196,81 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F8" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G8" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="H8" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>588.8</v>
+        <v>283.9</v>
       </c>
       <c r="J8" t="n">
-        <v>542.36</v>
+        <v>264.91</v>
       </c>
       <c r="K8" t="n">
-        <v>8.6</v>
+        <v>7.2</v>
       </c>
       <c r="L8" t="n">
-        <v>64.68000000000001</v>
+        <v>70.09</v>
       </c>
       <c r="M8" t="n">
-        <v>5.21</v>
+        <v>92.70999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>29-05-2026</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>0.474</v>
+        <v>3.303</v>
       </c>
       <c r="Q8" t="n">
-        <v>1098</v>
+        <v>2807</v>
       </c>
       <c r="R8" t="n">
-        <v>55.9</v>
+        <v>48.8</v>
       </c>
       <c r="S8" t="n">
-        <v>21</v>
+        <v>-3</v>
       </c>
       <c r="T8" t="n">
-        <v>-0.11</v>
+        <v>11</v>
       </c>
       <c r="U8" t="n">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="V8" t="n">
-        <v>-0.07000000000000001</v>
+        <v>1.05</v>
       </c>
       <c r="W8" t="n">
-        <v>1.58</v>
+        <v>29.6</v>
       </c>
       <c r="X8" t="n">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="Y8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z8" t="n">
-        <v>-110</v>
+        <v>24</v>
       </c>
       <c r="AA8" t="n">
-        <v>564.79</v>
+        <v>294.93</v>
       </c>
       <c r="AB8" t="n">
-        <v>495.72</v>
+        <v>279.96</v>
       </c>
       <c r="AC8" t="n">
-        <v>21.5</v>
+        <v>23.3</v>
       </c>
     </row>
     <row r="9">
@@ -1340,13 +1328,13 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>0.081</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="Q9" t="n">
-        <v>418</v>
+        <v>407</v>
       </c>
       <c r="R9" t="n">
-        <v>12.4</v>
+        <v>12</v>
       </c>
       <c r="S9" t="n">
         <v>-8</v>
@@ -1385,12 +1373,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>EUROPRATIK</t>
+          <t>STEL</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Euro Pratik Sales Limited</t>
+          <t>STEL HOLDINGS LIMITED</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1402,81 +1390,81 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F10" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G10" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="I10" t="n">
-        <v>283.9</v>
+        <v>588.8</v>
       </c>
       <c r="J10" t="n">
-        <v>266</v>
+        <v>556.59</v>
       </c>
       <c r="K10" t="n">
-        <v>6.7</v>
+        <v>5.8</v>
       </c>
       <c r="L10" t="n">
-        <v>70.09</v>
+        <v>64.68000000000001</v>
       </c>
       <c r="M10" t="n">
-        <v>153.77</v>
+        <v>4.12</v>
       </c>
       <c r="N10" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>29-05-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>5.245</v>
+        <v>0.38</v>
       </c>
       <c r="Q10" t="n">
-        <v>2932</v>
+        <v>1084</v>
       </c>
       <c r="R10" t="n">
-        <v>51</v>
+        <v>55.2</v>
       </c>
       <c r="S10" t="n">
-        <v>-3</v>
+        <v>21</v>
       </c>
       <c r="T10" t="n">
-        <v>11</v>
+        <v>-0.11</v>
       </c>
       <c r="U10" t="n">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="V10" t="n">
-        <v>1.05</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="W10" t="n">
-        <v>29.6</v>
+        <v>1.58</v>
       </c>
       <c r="X10" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="Y10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z10" t="n">
-        <v>24</v>
+        <v>-110</v>
       </c>
       <c r="AA10" t="n">
-        <v>294.93</v>
+        <v>564.79</v>
       </c>
       <c r="AB10" t="n">
-        <v>279.96</v>
+        <v>495.72</v>
       </c>
       <c r="AC10" t="n">
-        <v>23.3</v>
+        <v>21.5</v>
       </c>
     </row>
     <row r="11">
@@ -1534,13 +1522,13 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>0.438</v>
+        <v>0.455</v>
       </c>
       <c r="Q11" t="n">
-        <v>322</v>
+        <v>310</v>
       </c>
       <c r="R11" t="n">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="S11" t="n">
         <v>22</v>
@@ -1631,13 +1619,13 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>0.052</v>
+        <v>0.053</v>
       </c>
       <c r="Q12" t="n">
-        <v>801</v>
+        <v>794</v>
       </c>
       <c r="R12" t="n">
-        <v>85.59999999999999</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="S12" t="n">
         <v>15</v>
@@ -1676,16 +1664,16 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>INDIQUBE</t>
+          <t>CHEMBONDCH</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Indiqube Spaces Limited</t>
+          <t>CHEMBOND CHEMICALS LIMITED</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1693,94 +1681,96 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F13" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="G13" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="I13" t="n">
-        <v>178</v>
+        <v>264</v>
       </c>
       <c r="J13" t="n">
-        <v>164.1</v>
+        <v>230</v>
       </c>
       <c r="K13" t="n">
-        <v>8.5</v>
+        <v>14.8</v>
       </c>
       <c r="L13" t="n">
-        <v>60.6</v>
+        <v>67.65000000000001</v>
       </c>
       <c r="M13" t="n">
-        <v>0.25</v>
+        <v>0.7</v>
       </c>
       <c r="N13" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>24-06-2026</t>
+          <t>06-08-2026</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>0.007</v>
+        <v>0.097</v>
       </c>
       <c r="Q13" t="n">
-        <v>3780</v>
-      </c>
-      <c r="R13" t="inlineStr"/>
+        <v>720</v>
+      </c>
+      <c r="R13" t="n">
+        <v>60.1</v>
+      </c>
       <c r="S13" t="n">
-        <v>39</v>
+        <v>3</v>
       </c>
       <c r="T13" t="n">
-        <v>258</v>
+        <v>2.99</v>
       </c>
       <c r="U13" t="n">
-        <v>30</v>
+        <v>97</v>
       </c>
       <c r="V13" t="n">
-        <v>-1.13</v>
+        <v>1</v>
       </c>
       <c r="W13" t="n">
-        <v>6.38</v>
+        <v>11.6</v>
       </c>
       <c r="X13" t="n">
-        <v>10.11</v>
+        <v>0</v>
       </c>
       <c r="Y13" t="b">
         <v>1</v>
       </c>
       <c r="Z13" t="n">
-        <v>61</v>
+        <v>16.21</v>
       </c>
       <c r="AA13" t="n">
-        <v>171.3</v>
+        <v>228.71</v>
       </c>
       <c r="AB13" t="n">
-        <v>180</v>
+        <v>172.77</v>
       </c>
       <c r="AC13" t="n">
-        <v>0.5</v>
+        <v>66.3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TRUALT</t>
+          <t>INDIQUBE</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>TRUALT BIOENERGY LIMITED</t>
+          <t>Indiqube Spaces Limited</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1788,96 +1778,94 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="F14" t="n">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="G14" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>478</v>
+        <v>178</v>
       </c>
       <c r="J14" t="n">
-        <v>474.97</v>
+        <v>164.1</v>
       </c>
       <c r="K14" t="n">
-        <v>0.6</v>
+        <v>8.5</v>
       </c>
       <c r="L14" t="n">
-        <v>70.55</v>
+        <v>60.6</v>
       </c>
       <c r="M14" t="n">
-        <v>18.35</v>
+        <v>0.25</v>
       </c>
       <c r="N14" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>12-08-2026</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>0.446</v>
+        <v>0.006</v>
       </c>
       <c r="Q14" t="n">
-        <v>4111</v>
-      </c>
-      <c r="R14" t="n">
-        <v>28.8</v>
-      </c>
+        <v>3972</v>
+      </c>
+      <c r="R14" t="inlineStr"/>
       <c r="S14" t="n">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="T14" t="n">
-        <v>127</v>
+        <v>258</v>
       </c>
       <c r="U14" t="n">
-        <v>-14</v>
+        <v>30</v>
       </c>
       <c r="V14" t="n">
-        <v>6.41</v>
+        <v>-1.13</v>
       </c>
       <c r="W14" t="n">
-        <v>9.890000000000001</v>
+        <v>6.38</v>
       </c>
       <c r="X14" t="n">
-        <v>1.05</v>
+        <v>10.11</v>
       </c>
       <c r="Y14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z14" t="n">
-        <v>21</v>
+        <v>61</v>
       </c>
       <c r="AA14" t="n">
-        <v>460.31</v>
+        <v>171.3</v>
       </c>
       <c r="AB14" t="n">
-        <v>433.98</v>
+        <v>180</v>
       </c>
       <c r="AC14" t="n">
-        <v>8</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SENCO</t>
+          <t>TRUALT</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>SENCO GOLD LIMITED</t>
+          <t>TRUALT BIOENERGY LIMITED</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1885,81 +1873,81 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F15" t="n">
+        <v>5</v>
+      </c>
+      <c r="G15" t="n">
+        <v>25</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>478</v>
+      </c>
+      <c r="J15" t="n">
+        <v>474.82</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L15" t="n">
+        <v>70.55</v>
+      </c>
+      <c r="M15" t="n">
+        <v>10.22</v>
+      </c>
+      <c r="N15" t="n">
+        <v>5</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>12-08-2026</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>0.252</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>4061</v>
+      </c>
+      <c r="R15" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="S15" t="n">
+        <v>2</v>
+      </c>
+      <c r="T15" t="n">
+        <v>127</v>
+      </c>
+      <c r="U15" t="n">
+        <v>-14</v>
+      </c>
+      <c r="V15" t="n">
+        <v>6.41</v>
+      </c>
+      <c r="W15" t="n">
+        <v>9.890000000000001</v>
+      </c>
+      <c r="X15" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="Y15" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z15" t="n">
         <v>21</v>
       </c>
-      <c r="G15" t="n">
-        <v>15</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" t="n">
-        <v>342</v>
-      </c>
-      <c r="J15" t="n">
-        <v>334.88</v>
-      </c>
-      <c r="K15" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="L15" t="n">
-        <v>68.48</v>
-      </c>
-      <c r="M15" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="N15" t="n">
-        <v>1</v>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>30-06-2026</t>
-        </is>
-      </c>
-      <c r="P15" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>5602</v>
-      </c>
-      <c r="R15" t="n">
-        <v>9.470000000000001</v>
-      </c>
-      <c r="S15" t="n">
-        <v>43</v>
-      </c>
-      <c r="T15" t="n">
-        <v>223</v>
-      </c>
-      <c r="U15" t="n">
-        <v>175</v>
-      </c>
-      <c r="V15" t="n">
-        <v>6.97</v>
-      </c>
-      <c r="W15" t="n">
-        <v>21.4</v>
-      </c>
-      <c r="X15" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="Y15" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z15" t="n">
-        <v>7</v>
-      </c>
       <c r="AA15" t="n">
-        <v>360.79</v>
+        <v>460.31</v>
       </c>
       <c r="AB15" t="n">
-        <v>331.94</v>
+        <v>433.98</v>
       </c>
       <c r="AC15" t="n">
-        <v>-4.4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16">
@@ -2017,13 +2005,13 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>0.231</v>
+        <v>0.223</v>
       </c>
       <c r="Q16" t="n">
-        <v>1304</v>
+        <v>1347</v>
       </c>
       <c r="R16" t="n">
-        <v>45.5</v>
+        <v>47</v>
       </c>
       <c r="S16" t="n">
         <v>7</v>
@@ -2062,16 +2050,16 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>SENCO</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>HCL Technologies Limited</t>
+          <t>SENCO GOLD LIMITED</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -2079,193 +2067,193 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F17" t="n">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="G17" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>1325</v>
+        <v>342</v>
       </c>
       <c r="J17" t="n">
-        <v>1104.34</v>
+        <v>334.88</v>
       </c>
       <c r="K17" t="n">
-        <v>20</v>
+        <v>2.1</v>
       </c>
       <c r="L17" t="n">
-        <v>60.82</v>
+        <v>68.48</v>
       </c>
       <c r="M17" t="n">
-        <v>5.22</v>
+        <v>0.3</v>
       </c>
       <c r="N17" t="n">
         <v>1</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>12-06-2026</t>
+          <t>30-06-2026</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>0.001</v>
+        <v>0.005</v>
       </c>
       <c r="Q17" t="n">
-        <v>359561</v>
+        <v>5523</v>
       </c>
       <c r="R17" t="n">
-        <v>19.8</v>
+        <v>9.33</v>
       </c>
       <c r="S17" t="n">
+        <v>43</v>
+      </c>
+      <c r="T17" t="n">
+        <v>223</v>
+      </c>
+      <c r="U17" t="n">
+        <v>175</v>
+      </c>
+      <c r="V17" t="n">
+        <v>6.97</v>
+      </c>
+      <c r="W17" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="X17" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="Y17" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z17" t="n">
         <v>7</v>
       </c>
-      <c r="T17" t="n">
-        <v>4158</v>
-      </c>
-      <c r="U17" t="n">
-        <v>44</v>
-      </c>
-      <c r="V17" t="n">
-        <v>25.89</v>
-      </c>
-      <c r="W17" t="n">
-        <v>53.4</v>
-      </c>
-      <c r="X17" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="Y17" t="b">
-        <v>1</v>
-      </c>
-      <c r="Z17" t="n">
-        <v>29</v>
-      </c>
       <c r="AA17" t="n">
-        <v>1215.63</v>
+        <v>360.79</v>
       </c>
       <c r="AB17" t="n">
-        <v>1406.5</v>
+        <v>331.94</v>
       </c>
       <c r="AC17" t="n">
-        <v>-15.8</v>
+        <v>-4.4</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>LAOPALA</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>LA OPALA RG LIMITED</t>
+          <t>HCL Technologies Limited</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Watchlist</t>
+          <t>Buy on Breakout</t>
         </is>
       </c>
       <c r="E18" t="n">
+        <v>12</v>
+      </c>
+      <c r="F18" t="n">
+        <v>30</v>
+      </c>
+      <c r="G18" t="n">
+        <v>10</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>1325</v>
+      </c>
+      <c r="J18" t="n">
+        <v>1104.34</v>
+      </c>
+      <c r="K18" t="n">
         <v>20</v>
       </c>
-      <c r="F18" t="n">
-        <v>14</v>
-      </c>
-      <c r="G18" t="n">
-        <v>15</v>
-      </c>
-      <c r="H18" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" t="n">
-        <v>190.6</v>
-      </c>
-      <c r="J18" t="n">
-        <v>173.91</v>
-      </c>
-      <c r="K18" t="n">
-        <v>9.6</v>
-      </c>
       <c r="L18" t="n">
-        <v>65.64</v>
+        <v>60.82</v>
       </c>
       <c r="M18" t="n">
-        <v>2.61</v>
+        <v>5.22</v>
       </c>
       <c r="N18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>08-06-2026</t>
+          <t>12-06-2026</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>0.123</v>
+        <v>0.001</v>
       </c>
       <c r="Q18" t="n">
-        <v>2127</v>
+        <v>352074</v>
       </c>
       <c r="R18" t="n">
-        <v>22.5</v>
+        <v>19.4</v>
       </c>
       <c r="S18" t="n">
-        <v>-3</v>
+        <v>7</v>
       </c>
       <c r="T18" t="n">
-        <v>26</v>
+        <v>4158</v>
       </c>
       <c r="U18" t="n">
-        <v>-4</v>
+        <v>44</v>
       </c>
       <c r="V18" t="n">
-        <v>2.36</v>
+        <v>25.89</v>
       </c>
       <c r="W18" t="n">
-        <v>14.2</v>
+        <v>53.4</v>
       </c>
       <c r="X18" t="n">
-        <v>0.01</v>
+        <v>0.04</v>
       </c>
       <c r="Y18" t="b">
         <v>1</v>
       </c>
       <c r="Z18" t="n">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="AA18" t="n">
-        <v>184.16</v>
+        <v>1215.63</v>
       </c>
       <c r="AB18" t="n">
-        <v>193.41</v>
+        <v>1406.5</v>
       </c>
       <c r="AC18" t="n">
-        <v>-6.6</v>
+        <v>-15.8</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BAJAJHCARE</t>
+          <t>LAOPALA</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>BAJAJ HEALTHCARE LIMITED</t>
+          <t>LA OPALA RG LIMITED</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -2273,96 +2261,96 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F19" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="G19" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>323.05</v>
+        <v>190.6</v>
       </c>
       <c r="J19" t="n">
-        <v>297.3</v>
+        <v>173.91</v>
       </c>
       <c r="K19" t="n">
-        <v>8.699999999999999</v>
+        <v>9.6</v>
       </c>
       <c r="L19" t="n">
-        <v>67.69</v>
+        <v>65.64</v>
       </c>
       <c r="M19" t="n">
-        <v>2.97</v>
+        <v>2.61</v>
       </c>
       <c r="N19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>12-06-2026</t>
+          <t>08-06-2026</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>0.273</v>
+        <v>0.124</v>
       </c>
       <c r="Q19" t="n">
-        <v>1087</v>
+        <v>2105</v>
       </c>
       <c r="R19" t="n">
-        <v>19.3</v>
+        <v>22.3</v>
       </c>
       <c r="S19" t="n">
-        <v>12</v>
+        <v>-3</v>
       </c>
       <c r="T19" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="U19" t="n">
-        <v>20</v>
+        <v>-4</v>
       </c>
       <c r="V19" t="n">
-        <v>4.07</v>
+        <v>2.36</v>
       </c>
       <c r="W19" t="n">
-        <v>11.5</v>
+        <v>14.2</v>
       </c>
       <c r="X19" t="n">
-        <v>0.47</v>
+        <v>0.01</v>
       </c>
       <c r="Y19" t="b">
         <v>1</v>
       </c>
       <c r="Z19" t="n">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="AA19" t="n">
-        <v>329.31</v>
+        <v>184.16</v>
       </c>
       <c r="AB19" t="n">
-        <v>356.11</v>
+        <v>193.41</v>
       </c>
       <c r="AC19" t="n">
-        <v>-15</v>
+        <v>-6.6</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MOTOGENFIN</t>
+          <t>BAJAJHCARE</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>THE MOTOR &amp; GENERAL FINANCE LIMITED</t>
+          <t>BAJAJ HEALTHCARE LIMITED</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -2370,96 +2358,96 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="F20" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="G20" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="H20" t="n">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>26.07</v>
+        <v>323.05</v>
       </c>
       <c r="J20" t="n">
-        <v>29.18</v>
+        <v>297.3</v>
       </c>
       <c r="K20" t="n">
-        <v>-10.7</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="L20" t="n">
-        <v>69.03</v>
+        <v>67.69</v>
       </c>
       <c r="M20" t="n">
-        <v>1.48</v>
+        <v>2.97</v>
       </c>
       <c r="N20" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>12-06-2026</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>1.465</v>
+        <v>0.274</v>
       </c>
       <c r="Q20" t="n">
-        <v>101</v>
+        <v>1085</v>
       </c>
       <c r="R20" t="n">
-        <v>72.59999999999999</v>
+        <v>19.3</v>
       </c>
       <c r="S20" t="n">
-        <v>-1</v>
+        <v>12</v>
       </c>
       <c r="T20" t="n">
-        <v>0.4</v>
+        <v>29</v>
       </c>
       <c r="U20" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="V20" t="n">
-        <v>0.59</v>
+        <v>4.07</v>
       </c>
       <c r="W20" t="n">
-        <v>-0.18</v>
+        <v>11.5</v>
       </c>
       <c r="X20" t="n">
-        <v>0</v>
+        <v>0.47</v>
       </c>
       <c r="Y20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z20" t="n">
-        <v>21.51</v>
+        <v>17</v>
       </c>
       <c r="AA20" t="n">
-        <v>27.94</v>
+        <v>329.31</v>
       </c>
       <c r="AB20" t="n">
-        <v>24.6</v>
+        <v>356.11</v>
       </c>
       <c r="AC20" t="n">
-        <v>14</v>
+        <v>-15</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BMWVENTLTD</t>
+          <t>GANESHCP</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>BMW VENTURES LIMITED</t>
+          <t>GANESH CONSUMER PRODUCTS LIMITED</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -2467,96 +2455,96 @@
         </is>
       </c>
       <c r="E21" t="n">
+        <v>20</v>
+      </c>
+      <c r="F21" t="n">
         <v>25</v>
       </c>
-      <c r="F21" t="n">
-        <v>23</v>
-      </c>
       <c r="G21" t="n">
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>57.32</v>
+        <v>164.67</v>
       </c>
       <c r="J21" t="n">
-        <v>60.13</v>
+        <v>204.13</v>
       </c>
       <c r="K21" t="n">
-        <v>-4.7</v>
+        <v>-19.3</v>
       </c>
       <c r="L21" t="n">
-        <v>73.01000000000001</v>
+        <v>64.08</v>
       </c>
       <c r="M21" t="n">
-        <v>1.41</v>
+        <v>7.57</v>
       </c>
       <c r="N21" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>06-08-2026</t>
+          <t>30-06-2026</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>0.281</v>
+        <v>1.132</v>
       </c>
       <c r="Q21" t="n">
-        <v>501</v>
+        <v>669</v>
       </c>
       <c r="R21" t="n">
-        <v>12.5</v>
+        <v>14.8</v>
       </c>
       <c r="S21" t="n">
-        <v>19</v>
+        <v>-1</v>
       </c>
       <c r="T21" t="n">
         <v>21</v>
       </c>
       <c r="U21" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="V21" t="n">
-        <v>1.22</v>
+        <v>3.1</v>
       </c>
       <c r="W21" t="n">
-        <v>12</v>
+        <v>19.4</v>
       </c>
       <c r="X21" t="n">
-        <v>0.58</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Y21" t="b">
         <v>1</v>
       </c>
       <c r="Z21" t="n">
-        <v>3.4</v>
+        <v>11</v>
       </c>
       <c r="AA21" t="n">
-        <v>58.33</v>
+        <v>184.08</v>
       </c>
       <c r="AB21" t="n">
-        <v>59.71</v>
+        <v>205.91</v>
       </c>
       <c r="AC21" t="n">
-        <v>-2.3</v>
+        <v>-17</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>GANESHCP</t>
+          <t>ARSSBL</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>GANESH CONSUMER PRODUCTS LIMITED</t>
+          <t>Anand Rathi Share and Stock Brokers Limited</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2564,10 +2552,10 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F22" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
@@ -2576,84 +2564,84 @@
         <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>164.67</v>
+        <v>511.95</v>
       </c>
       <c r="J22" t="n">
-        <v>204.13</v>
+        <v>545.03</v>
       </c>
       <c r="K22" t="n">
-        <v>-19.3</v>
+        <v>-6.1</v>
       </c>
       <c r="L22" t="n">
-        <v>64.08</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="M22" t="n">
-        <v>7.57</v>
+        <v>1.09</v>
       </c>
       <c r="N22" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>30-06-2026</t>
+          <t>16-06-2026</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>1.145</v>
+        <v>0.034</v>
       </c>
       <c r="Q22" t="n">
-        <v>661</v>
+        <v>3228</v>
       </c>
       <c r="R22" t="n">
-        <v>14.6</v>
+        <v>21.9</v>
       </c>
       <c r="S22" t="n">
-        <v>-1</v>
+        <v>17</v>
       </c>
       <c r="T22" t="n">
-        <v>21</v>
+        <v>97</v>
       </c>
       <c r="U22" t="n">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="V22" t="n">
-        <v>3.1</v>
+        <v>3.73</v>
       </c>
       <c r="W22" t="n">
-        <v>19.4</v>
+        <v>19.8</v>
       </c>
       <c r="X22" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.62</v>
       </c>
       <c r="Y22" t="b">
         <v>1</v>
       </c>
       <c r="Z22" t="n">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="AA22" t="n">
-        <v>184.08</v>
+        <v>534.05</v>
       </c>
       <c r="AB22" t="n">
-        <v>205.91</v>
+        <v>563.1</v>
       </c>
       <c r="AC22" t="n">
-        <v>-17</v>
+        <v>-12.4</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ARSSBL</t>
+          <t>AJMERA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Anand Rathi Share and Stock Brokers Limited</t>
+          <t>AJMERA REALTY &amp; INFRA INDIA LIMITED</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -2661,81 +2649,81 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F23" t="n">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>511.95</v>
+        <v>119.6</v>
       </c>
       <c r="J23" t="n">
-        <v>545.03</v>
+        <v>114.86</v>
       </c>
       <c r="K23" t="n">
-        <v>-6.1</v>
+        <v>4.1</v>
       </c>
       <c r="L23" t="n">
-        <v>69.90000000000001</v>
+        <v>69.73999999999999</v>
       </c>
       <c r="M23" t="n">
-        <v>2.18</v>
+        <v>7.36</v>
       </c>
       <c r="N23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>16-06-2026</t>
+          <t>04-06-2026</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>0.068</v>
+        <v>0.321</v>
       </c>
       <c r="Q23" t="n">
-        <v>3211</v>
+        <v>2296</v>
       </c>
       <c r="R23" t="n">
-        <v>21.8</v>
+        <v>19.7</v>
       </c>
       <c r="S23" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="T23" t="n">
-        <v>97</v>
+        <v>46</v>
       </c>
       <c r="U23" t="n">
-        <v>53</v>
+        <v>-4</v>
       </c>
       <c r="V23" t="n">
-        <v>3.73</v>
+        <v>1.17</v>
       </c>
       <c r="W23" t="n">
-        <v>19.8</v>
+        <v>14.2</v>
       </c>
       <c r="X23" t="n">
-        <v>0.62</v>
+        <v>0.46</v>
       </c>
       <c r="Y23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z23" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="AA23" t="n">
-        <v>534.05</v>
+        <v>127.67</v>
       </c>
       <c r="AB23" t="n">
-        <v>563.1</v>
+        <v>369.15</v>
       </c>
       <c r="AC23" t="n">
-        <v>-12.4</v>
+        <v>-21.7</v>
       </c>
     </row>
     <row r="24">
@@ -2796,7 +2784,7 @@
         <v>0.097</v>
       </c>
       <c r="Q24" t="n">
-        <v>1524</v>
+        <v>1525</v>
       </c>
       <c r="R24" t="n">
         <v>13.8</v>
@@ -2838,16 +2826,16 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AJMERA</t>
+          <t>MOTOGENFIN</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>AJMERA REALTY &amp; INFRA INDIA LIMITED</t>
+          <t>THE MOTOR &amp; GENERAL FINANCE LIMITED</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -2855,81 +2843,77 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F25" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G25" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="I25" t="n">
-        <v>119.6</v>
+        <v>26.07</v>
       </c>
       <c r="J25" t="n">
-        <v>114.86</v>
+        <v>29.14</v>
       </c>
       <c r="K25" t="n">
-        <v>4.1</v>
+        <v>-10.5</v>
       </c>
       <c r="L25" t="n">
-        <v>69.73999999999999</v>
+        <v>69.03</v>
       </c>
       <c r="M25" t="n">
-        <v>7.36</v>
+        <v>1.34</v>
       </c>
       <c r="N25" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>04-06-2026</t>
-        </is>
-      </c>
-      <c r="P25" t="n">
-        <v>0.315</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>2337</v>
-      </c>
+          <t>25-06-2026</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
       <c r="R25" t="n">
-        <v>20.1</v>
+        <v>71.3</v>
       </c>
       <c r="S25" t="n">
-        <v>18</v>
+        <v>-1</v>
       </c>
       <c r="T25" t="n">
-        <v>46</v>
+        <v>0.4</v>
       </c>
       <c r="U25" t="n">
-        <v>-4</v>
+        <v>26</v>
       </c>
       <c r="V25" t="n">
-        <v>1.17</v>
+        <v>0.59</v>
       </c>
       <c r="W25" t="n">
-        <v>14.2</v>
+        <v>-0.18</v>
       </c>
       <c r="X25" t="n">
-        <v>0.46</v>
+        <v>0</v>
       </c>
       <c r="Y25" t="b">
         <v>0</v>
       </c>
       <c r="Z25" t="n">
-        <v>38</v>
+        <v>21.51</v>
       </c>
       <c r="AA25" t="n">
-        <v>127.67</v>
+        <v>27.94</v>
       </c>
       <c r="AB25" t="n">
-        <v>369.15</v>
+        <v>24.6</v>
       </c>
       <c r="AC25" t="n">
-        <v>-21.7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="26">
@@ -2987,13 +2971,13 @@
         </is>
       </c>
       <c r="P26" t="n">
-        <v>0.176</v>
+        <v>0.175</v>
       </c>
       <c r="Q26" t="n">
-        <v>705</v>
+        <v>709</v>
       </c>
       <c r="R26" t="n">
-        <v>12.8</v>
+        <v>12.9</v>
       </c>
       <c r="S26" t="n">
         <v>185</v>
@@ -3080,13 +3064,13 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>0.172</v>
+        <v>0.173</v>
       </c>
       <c r="Q27" t="n">
-        <v>2318</v>
+        <v>2310</v>
       </c>
       <c r="R27" t="n">
-        <v>19</v>
+        <v>18.9</v>
       </c>
       <c r="S27" t="n">
         <v>8</v>
@@ -3125,12 +3109,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>OMPOWER</t>
+          <t>THOMASCOOK</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Om Power Transmission Limited</t>
+          <t>THOMAS COOK (INDIA) LIMITED</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3142,10 +3126,10 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F28" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
@@ -3154,78 +3138,80 @@
         <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>167.95</v>
+        <v>103.75</v>
       </c>
       <c r="J28" t="n">
-        <v>182.69</v>
+        <v>109.31</v>
       </c>
       <c r="K28" t="n">
-        <v>-8.1</v>
+        <v>-5.1</v>
       </c>
       <c r="L28" t="n">
-        <v>69.05</v>
+        <v>72.34</v>
       </c>
       <c r="M28" t="n">
-        <v>0.74</v>
+        <v>48.4</v>
       </c>
       <c r="N28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>24-06-2026</t>
+          <t>11-06-2026</t>
         </is>
       </c>
       <c r="P28" t="n">
-        <v>0.128</v>
+        <v>1.006</v>
       </c>
       <c r="Q28" t="n">
-        <v>578</v>
+        <v>4813</v>
       </c>
       <c r="R28" t="n">
-        <v>13.7</v>
+        <v>38.6</v>
       </c>
       <c r="S28" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="T28" t="n">
-        <v>15</v>
+        <v>42</v>
       </c>
       <c r="U28" t="n">
-        <v>82</v>
+        <v>8</v>
       </c>
       <c r="V28" t="n">
-        <v>3.07</v>
+        <v>1.25</v>
       </c>
       <c r="W28" t="n">
-        <v>42.7</v>
+        <v>9.69</v>
       </c>
       <c r="X28" t="n">
-        <v>0.35</v>
+        <v>0.06</v>
       </c>
       <c r="Y28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z28" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="AA28" t="n">
-        <v>173.7</v>
-      </c>
-      <c r="AB28" t="inlineStr"/>
+        <v>106.03</v>
+      </c>
+      <c r="AB28" t="n">
+        <v>116.69</v>
+      </c>
       <c r="AC28" t="n">
-        <v>-13.1</v>
+        <v>-9.9</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>THOMASCOOK</t>
+          <t>OMPOWER</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>THOMAS COOK (INDIA) LIMITED</t>
+          <t>Om Power Transmission Limited</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3237,10 +3223,10 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F29" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="G29" t="n">
         <v>0</v>
@@ -3249,69 +3235,67 @@
         <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>103.75</v>
+        <v>167.95</v>
       </c>
       <c r="J29" t="n">
-        <v>109.31</v>
+        <v>182.69</v>
       </c>
       <c r="K29" t="n">
-        <v>-5.1</v>
+        <v>-8.1</v>
       </c>
       <c r="L29" t="n">
-        <v>72.34</v>
+        <v>69.05</v>
       </c>
       <c r="M29" t="n">
-        <v>48.4</v>
+        <v>0.74</v>
       </c>
       <c r="N29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>11-06-2026</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="P29" t="n">
-        <v>0.992</v>
+        <v>0.129</v>
       </c>
       <c r="Q29" t="n">
-        <v>4878</v>
+        <v>573</v>
       </c>
       <c r="R29" t="n">
-        <v>39.1</v>
+        <v>13.6</v>
       </c>
       <c r="S29" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="T29" t="n">
-        <v>42</v>
+        <v>15</v>
       </c>
       <c r="U29" t="n">
-        <v>8</v>
+        <v>82</v>
       </c>
       <c r="V29" t="n">
-        <v>1.25</v>
+        <v>3.07</v>
       </c>
       <c r="W29" t="n">
-        <v>9.69</v>
+        <v>42.7</v>
       </c>
       <c r="X29" t="n">
-        <v>0.06</v>
+        <v>0.35</v>
       </c>
       <c r="Y29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z29" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="AA29" t="n">
-        <v>106.03</v>
-      </c>
-      <c r="AB29" t="n">
-        <v>116.69</v>
-      </c>
+        <v>173.7</v>
+      </c>
+      <c r="AB29" t="inlineStr"/>
       <c r="AC29" t="n">
-        <v>-9.9</v>
+        <v>-13.1</v>
       </c>
     </row>
     <row r="30">
@@ -3369,13 +3353,13 @@
         </is>
       </c>
       <c r="P30" t="n">
-        <v>0.172</v>
+        <v>0.17</v>
       </c>
       <c r="Q30" t="n">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="R30" t="n">
-        <v>1182</v>
+        <v>1198</v>
       </c>
       <c r="S30" t="n">
         <v>-61</v>
@@ -3410,16 +3394,16 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>GRMOVER</t>
+          <t>BMWVENTLTD</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>GRM OVERSEAS LIMITED</t>
+          <t>BMW VENTURES LIMITED</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -3427,96 +3411,96 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F31" t="n">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="G31" t="n">
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="I31" t="n">
-        <v>90</v>
+        <v>57.32</v>
       </c>
       <c r="J31" t="n">
-        <v>100.13</v>
+        <v>60.15</v>
       </c>
       <c r="K31" t="n">
-        <v>-10.1</v>
+        <v>-4.7</v>
       </c>
       <c r="L31" t="n">
-        <v>71.72</v>
+        <v>73.01000000000001</v>
       </c>
       <c r="M31" t="n">
-        <v>15.9</v>
+        <v>0.9</v>
       </c>
       <c r="N31" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>24-06-2026</t>
+          <t>06-08-2026</t>
         </is>
       </c>
       <c r="P31" t="n">
-        <v>0.868</v>
+        <v>0.184</v>
       </c>
       <c r="Q31" t="n">
-        <v>1831</v>
+        <v>489</v>
       </c>
       <c r="R31" t="n">
-        <v>33.1</v>
+        <v>12.2</v>
       </c>
       <c r="S31" t="n">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="T31" t="n">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="U31" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="V31" t="n">
-        <v>0.9</v>
+        <v>1.22</v>
       </c>
       <c r="W31" t="n">
-        <v>11.3</v>
+        <v>12</v>
       </c>
       <c r="X31" t="n">
-        <v>0.67</v>
+        <v>0.58</v>
       </c>
       <c r="Y31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z31" t="n">
-        <v>9</v>
+        <v>3.4</v>
       </c>
       <c r="AA31" t="n">
-        <v>92.88</v>
+        <v>58.33</v>
       </c>
       <c r="AB31" t="n">
-        <v>206.69</v>
+        <v>59.71</v>
       </c>
       <c r="AC31" t="n">
-        <v>-45.3</v>
+        <v>-2.3</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>MANINFRA</t>
+          <t>GRMOVER</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MAN INFRACONSTRUCTION LIMITED</t>
+          <t>GRM OVERSEAS LIMITED</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -3524,10 +3508,10 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F32" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="G32" t="n">
         <v>0</v>
@@ -3536,69 +3520,69 @@
         <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="J32" t="n">
-        <v>105.19</v>
+        <v>95.54000000000001</v>
       </c>
       <c r="K32" t="n">
-        <v>-1.1</v>
+        <v>-5.8</v>
       </c>
       <c r="L32" t="n">
-        <v>67.15000000000001</v>
+        <v>71.72</v>
       </c>
       <c r="M32" t="n">
-        <v>7.89</v>
+        <v>10.87</v>
       </c>
       <c r="N32" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="P32" t="n">
-        <v>0.187</v>
+        <v>0.599</v>
       </c>
       <c r="Q32" t="n">
-        <v>4210</v>
+        <v>1815</v>
       </c>
       <c r="R32" t="n">
-        <v>27.4</v>
+        <v>32.8</v>
       </c>
       <c r="S32" t="n">
-        <v>-25</v>
+        <v>39</v>
       </c>
       <c r="T32" t="n">
-        <v>71</v>
+        <v>31</v>
       </c>
       <c r="U32" t="n">
-        <v>-11</v>
+        <v>8</v>
       </c>
       <c r="V32" t="n">
-        <v>1.48</v>
+        <v>0.9</v>
       </c>
       <c r="W32" t="n">
-        <v>10.7</v>
+        <v>11.3</v>
       </c>
       <c r="X32" t="n">
-        <v>0</v>
+        <v>0.67</v>
       </c>
       <c r="Y32" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z32" t="n">
-        <v>69</v>
+        <v>9</v>
       </c>
       <c r="AA32" t="n">
-        <v>105.07</v>
+        <v>92.88</v>
       </c>
       <c r="AB32" t="n">
-        <v>113.83</v>
+        <v>206.69</v>
       </c>
       <c r="AC32" t="n">
-        <v>-16.2</v>
+        <v>-45.3</v>
       </c>
     </row>
     <row r="33">
@@ -3636,19 +3620,19 @@
         <v>74.34999999999999</v>
       </c>
       <c r="J33" t="n">
-        <v>74.84999999999999</v>
+        <v>74.92</v>
       </c>
       <c r="K33" t="n">
-        <v>-0.7</v>
+        <v>-0.8</v>
       </c>
       <c r="L33" t="n">
         <v>62.78</v>
       </c>
       <c r="M33" t="n">
-        <v>1.8</v>
+        <v>1.48</v>
       </c>
       <c r="N33" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -3656,13 +3640,13 @@
         </is>
       </c>
       <c r="P33" t="n">
-        <v>0.474</v>
+        <v>0.389</v>
       </c>
       <c r="Q33" t="n">
         <v>380</v>
       </c>
       <c r="R33" t="n">
-        <v>35.3</v>
+        <v>35.2</v>
       </c>
       <c r="S33" t="n">
         <v>21</v>
@@ -3753,10 +3737,10 @@
         </is>
       </c>
       <c r="P34" t="n">
-        <v>0.549</v>
+        <v>0.544</v>
       </c>
       <c r="Q34" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="R34" t="inlineStr"/>
       <c r="S34" t="n">
@@ -3854,7 +3838,7 @@
         <v>384</v>
       </c>
       <c r="R35" t="n">
-        <v>95</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="S35" t="n">
         <v>246</v>
@@ -3925,19 +3909,19 @@
         <v>285</v>
       </c>
       <c r="J36" t="n">
-        <v>297.22</v>
+        <v>292.28</v>
       </c>
       <c r="K36" t="n">
-        <v>-4.1</v>
+        <v>-2.5</v>
       </c>
       <c r="L36" t="n">
         <v>70.45</v>
       </c>
       <c r="M36" t="n">
-        <v>1.9</v>
+        <v>1.29</v>
       </c>
       <c r="N36" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -3945,10 +3929,10 @@
         </is>
       </c>
       <c r="P36" t="n">
-        <v>0.117</v>
+        <v>0.08</v>
       </c>
       <c r="Q36" t="n">
-        <v>1621</v>
+        <v>1622</v>
       </c>
       <c r="R36" t="n">
         <v>20.6</v>
@@ -3990,113 +3974,113 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>VSTL</t>
+          <t>MANINFRA</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>VIBHOR STEEL TUBES LIMITED</t>
+          <t>MAN INFRACONSTRUCTION LIMITED</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Avoid</t>
+          <t>Fundamental Watch</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F37" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G37" t="n">
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>106.8</v>
+        <v>104</v>
       </c>
       <c r="J37" t="n">
-        <v>117.88</v>
+        <v>105.19</v>
       </c>
       <c r="K37" t="n">
-        <v>-9.4</v>
+        <v>-1.1</v>
       </c>
       <c r="L37" t="n">
-        <v>73.48</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="M37" t="n">
-        <v>0.27</v>
+        <v>2.63</v>
       </c>
       <c r="N37" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>12-06-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
       <c r="P37" t="n">
-        <v>0.132</v>
+        <v>0.061</v>
       </c>
       <c r="Q37" t="n">
-        <v>204</v>
+        <v>4280</v>
       </c>
       <c r="R37" t="n">
-        <v>24.2</v>
+        <v>27.9</v>
       </c>
       <c r="S37" t="n">
-        <v>21</v>
+        <v>-25</v>
       </c>
       <c r="T37" t="n">
-        <v>12.07</v>
+        <v>71</v>
       </c>
       <c r="U37" t="n">
-        <v>-29</v>
+        <v>-11</v>
       </c>
       <c r="V37" t="n">
-        <v>1.02</v>
+        <v>1.48</v>
       </c>
       <c r="W37" t="n">
-        <v>7.92</v>
+        <v>10.7</v>
       </c>
       <c r="X37" t="n">
-        <v>0.98</v>
+        <v>0</v>
       </c>
       <c r="Y37" t="b">
         <v>1</v>
       </c>
       <c r="Z37" t="n">
-        <v>4.11</v>
+        <v>69</v>
       </c>
       <c r="AA37" t="n">
-        <v>113.29</v>
+        <v>105.07</v>
       </c>
       <c r="AB37" t="n">
-        <v>121.76</v>
+        <v>113.83</v>
       </c>
       <c r="AC37" t="n">
-        <v>-10.9</v>
+        <v>-16.2</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>WCIL</t>
+          <t>VSTL</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>WESTERN CARRIERS (INDIA) LIMITED</t>
+          <t>VIBHOR STEEL TUBES LIMITED</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -4107,7 +4091,7 @@
         <v>20</v>
       </c>
       <c r="F38" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G38" t="n">
         <v>0</v>
@@ -4116,84 +4100,84 @@
         <v>-2</v>
       </c>
       <c r="I38" t="n">
-        <v>87.98</v>
+        <v>106.8</v>
       </c>
       <c r="J38" t="n">
-        <v>100.33</v>
+        <v>117.88</v>
       </c>
       <c r="K38" t="n">
-        <v>-12.3</v>
+        <v>-9.4</v>
       </c>
       <c r="L38" t="n">
-        <v>71.89</v>
+        <v>73.48</v>
       </c>
       <c r="M38" t="n">
-        <v>0.63</v>
+        <v>0.27</v>
       </c>
       <c r="N38" t="n">
         <v>5</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>30-06-2026</t>
+          <t>12-06-2026</t>
         </is>
       </c>
       <c r="P38" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.136</v>
       </c>
       <c r="Q38" t="n">
-        <v>893</v>
+        <v>199</v>
       </c>
       <c r="R38" t="n">
-        <v>24.3</v>
+        <v>23.6</v>
       </c>
       <c r="S38" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="T38" t="n">
-        <v>18.68</v>
+        <v>12.07</v>
       </c>
       <c r="U38" t="n">
-        <v>-36</v>
+        <v>-29</v>
       </c>
       <c r="V38" t="n">
-        <v>0.85</v>
+        <v>1.02</v>
       </c>
       <c r="W38" t="n">
-        <v>6.79</v>
+        <v>7.92</v>
       </c>
       <c r="X38" t="n">
-        <v>0.26</v>
+        <v>0.98</v>
       </c>
       <c r="Y38" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z38" t="n">
-        <v>4.02</v>
+        <v>4.11</v>
       </c>
       <c r="AA38" t="n">
-        <v>94.26000000000001</v>
+        <v>113.29</v>
       </c>
       <c r="AB38" t="n">
-        <v>106.34</v>
+        <v>121.76</v>
       </c>
       <c r="AC38" t="n">
-        <v>-27.3</v>
+        <v>-10.9</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>TIGERLOGS</t>
+          <t>WCIL</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Tiger Logistics (India) Limited</t>
+          <t>WESTERN CARRIERS (INDIA) LIMITED</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -4201,10 +4185,10 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F39" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G39" t="n">
         <v>0</v>
@@ -4213,68 +4197,165 @@
         <v>-2</v>
       </c>
       <c r="I39" t="n">
+        <v>87.98</v>
+      </c>
+      <c r="J39" t="n">
+        <v>100.33</v>
+      </c>
+      <c r="K39" t="n">
+        <v>-12.3</v>
+      </c>
+      <c r="L39" t="n">
+        <v>71.89</v>
+      </c>
+      <c r="M39" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="N39" t="n">
+        <v>5</v>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>30-06-2026</t>
+        </is>
+      </c>
+      <c r="P39" t="n">
+        <v>0.07099999999999999</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>882</v>
+      </c>
+      <c r="R39" t="n">
+        <v>24</v>
+      </c>
+      <c r="S39" t="n">
+        <v>9</v>
+      </c>
+      <c r="T39" t="n">
+        <v>18.68</v>
+      </c>
+      <c r="U39" t="n">
+        <v>-36</v>
+      </c>
+      <c r="V39" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="W39" t="n">
+        <v>6.79</v>
+      </c>
+      <c r="X39" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="Y39" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z39" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="AA39" t="n">
+        <v>94.26000000000001</v>
+      </c>
+      <c r="AB39" t="n">
+        <v>106.34</v>
+      </c>
+      <c r="AC39" t="n">
+        <v>-27.3</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>TIGERLOGS</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Tiger Logistics (India) Limited</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>25</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>15</v>
+      </c>
+      <c r="F40" t="n">
+        <v>12</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" t="n">
+        <v>-2</v>
+      </c>
+      <c r="I40" t="n">
         <v>26.8</v>
       </c>
-      <c r="J39" t="n">
+      <c r="J40" t="n">
         <v>36.7</v>
       </c>
-      <c r="K39" t="n">
+      <c r="K40" t="n">
         <v>-27</v>
       </c>
-      <c r="L39" t="n">
+      <c r="L40" t="n">
         <v>61.81</v>
       </c>
-      <c r="M39" t="n">
+      <c r="M40" t="n">
         <v>0.66</v>
       </c>
-      <c r="N39" t="n">
+      <c r="N40" t="n">
         <v>10</v>
       </c>
-      <c r="O39" t="inlineStr">
+      <c r="O40" t="inlineStr">
         <is>
           <t>30-06-2026</t>
         </is>
       </c>
-      <c r="P39" t="n">
-        <v>0.232</v>
-      </c>
-      <c r="Q39" t="n">
-        <v>285</v>
-      </c>
-      <c r="R39" t="n">
-        <v>15</v>
-      </c>
-      <c r="S39" t="n">
+      <c r="P40" t="n">
+        <v>0.223</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>296</v>
+      </c>
+      <c r="R40" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="S40" t="n">
         <v>16</v>
       </c>
-      <c r="T39" t="n">
+      <c r="T40" t="n">
         <v>2.79</v>
       </c>
-      <c r="U39" t="n">
+      <c r="U40" t="n">
         <v>-30</v>
       </c>
-      <c r="V39" t="n">
+      <c r="V40" t="n">
         <v>0.21</v>
       </c>
-      <c r="W39" t="n">
+      <c r="W40" t="n">
         <v>17.6</v>
       </c>
-      <c r="X39" t="n">
+      <c r="X40" t="n">
         <v>0.31</v>
       </c>
-      <c r="Y39" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z39" t="n">
+      <c r="Y40" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z40" t="n">
         <v>1.83</v>
       </c>
-      <c r="AA39" t="n">
+      <c r="AA40" t="n">
         <v>32.24</v>
       </c>
-      <c r="AB39" t="n">
+      <c r="AB40" t="n">
         <v>33.9</v>
       </c>
-      <c r="AC39" t="n">
+      <c r="AC40" t="n">
         <v>-20.4</v>
       </c>
     </row>
@@ -4289,7 +4370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4304,47 +4385,47 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Symbol</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>CompanyName</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>LastPrice</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>AvgPrice</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>PriceDiffPct</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>PromoHolding</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>ValueCr</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>NumBuyTxn</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>acqtoDt</t>
         </is>
@@ -4388,140 +4469,140 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MACPOWER</t>
+          <t>PREMIERPOL</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MACPOWER CNC MACHINES LIMITED</t>
+          <t>PREMIER POLYFILM LIMITED</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1798</v>
+        <v>85.45</v>
       </c>
       <c r="D3" t="n">
-        <v>920.51</v>
+        <v>54.77</v>
       </c>
       <c r="E3" t="n">
-        <v>95.3</v>
+        <v>56</v>
       </c>
       <c r="F3" t="n">
-        <v>73.16</v>
+        <v>67.45999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>0.44</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>04-06-2026</t>
+          <t>17-06-2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>APLLTD</t>
+          <t>MACPOWER</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Alembic Pharmaceuticals Limited</t>
+          <t>MACPOWER CNC MACHINES LIMITED</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>823.8</v>
+        <v>1798</v>
       </c>
       <c r="D4" t="n">
-        <v>754.37</v>
+        <v>920.51</v>
       </c>
       <c r="E4" t="n">
-        <v>9.199999999999999</v>
+        <v>95.3</v>
       </c>
       <c r="F4" t="n">
-        <v>69.61</v>
+        <v>73.16</v>
       </c>
       <c r="G4" t="n">
-        <v>24.22</v>
+        <v>0.44</v>
       </c>
       <c r="H4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>04-06-2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>THANGAMAYL</t>
+          <t>APLLTD</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>THANGAMAYIL JEWELLERY LIMITED</t>
+          <t>Alembic Pharmaceuticals Limited</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>5329</v>
+        <v>823.8</v>
       </c>
       <c r="D5" t="n">
-        <v>5085.36</v>
+        <v>753.55</v>
       </c>
       <c r="E5" t="n">
-        <v>4.8</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="F5" t="n">
-        <v>67.16</v>
+        <v>69.61</v>
       </c>
       <c r="G5" t="n">
-        <v>5.22</v>
+        <v>19.68</v>
       </c>
       <c r="H5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>07-08-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CHEMBONDCH</t>
+          <t>THANGAMAYL</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CHEMBOND CHEMICALS LIMITED</t>
+          <t>THANGAMAYIL JEWELLERY LIMITED</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>264</v>
+        <v>5329</v>
       </c>
       <c r="D6" t="n">
-        <v>230</v>
+        <v>5085.36</v>
       </c>
       <c r="E6" t="n">
-        <v>14.8</v>
+        <v>4.8</v>
       </c>
       <c r="F6" t="n">
-        <v>67.65000000000001</v>
+        <v>67.16</v>
       </c>
       <c r="G6" t="n">
-        <v>1.4</v>
+        <v>5.22</v>
       </c>
       <c r="H6" t="n">
         <v>4</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>06-08-2026</t>
+          <t>07-08-2026</t>
         </is>
       </c>
     </row>
@@ -4540,10 +4621,10 @@
         <v>576</v>
       </c>
       <c r="D7" t="n">
-        <v>374.61</v>
+        <v>379.74</v>
       </c>
       <c r="E7" t="n">
-        <v>53.8</v>
+        <v>51.7</v>
       </c>
       <c r="F7" t="n">
         <v>63.09</v>
@@ -4552,7 +4633,7 @@
         <v>13.87</v>
       </c>
       <c r="H7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -4563,35 +4644,35 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>STEL</t>
+          <t>EUROPRATIK</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>STEL HOLDINGS LIMITED</t>
+          <t>Euro Pratik Sales Limited</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>588.8</v>
+        <v>283.9</v>
       </c>
       <c r="D8" t="n">
-        <v>542.36</v>
+        <v>264.91</v>
       </c>
       <c r="E8" t="n">
-        <v>8.6</v>
+        <v>7.2</v>
       </c>
       <c r="F8" t="n">
-        <v>64.68000000000001</v>
+        <v>70.09</v>
       </c>
       <c r="G8" t="n">
-        <v>5.21</v>
+        <v>92.70999999999999</v>
       </c>
       <c r="H8" t="n">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>29-05-2026</t>
         </is>
       </c>
     </row>
@@ -4633,35 +4714,35 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>EUROPRATIK</t>
+          <t>STEL</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Euro Pratik Sales Limited</t>
+          <t>STEL HOLDINGS LIMITED</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>283.9</v>
+        <v>588.8</v>
       </c>
       <c r="D10" t="n">
-        <v>266</v>
+        <v>556.59</v>
       </c>
       <c r="E10" t="n">
-        <v>6.7</v>
+        <v>5.8</v>
       </c>
       <c r="F10" t="n">
-        <v>70.09</v>
+        <v>64.68000000000001</v>
       </c>
       <c r="G10" t="n">
-        <v>153.77</v>
+        <v>4.12</v>
       </c>
       <c r="H10" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>29-05-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
     </row>
@@ -4738,105 +4819,105 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>INDIQUBE</t>
+          <t>CHEMBONDCH</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Indiqube Spaces Limited</t>
+          <t>CHEMBOND CHEMICALS LIMITED</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>178</v>
+        <v>264</v>
       </c>
       <c r="D13" t="n">
-        <v>164.1</v>
+        <v>230</v>
       </c>
       <c r="E13" t="n">
-        <v>8.5</v>
+        <v>14.8</v>
       </c>
       <c r="F13" t="n">
-        <v>60.6</v>
+        <v>67.65000000000001</v>
       </c>
       <c r="G13" t="n">
-        <v>0.25</v>
+        <v>0.7</v>
       </c>
       <c r="H13" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>24-06-2026</t>
+          <t>06-08-2026</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TRUALT</t>
+          <t>INDIQUBE</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>TRUALT BIOENERGY LIMITED</t>
+          <t>Indiqube Spaces Limited</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>478</v>
+        <v>178</v>
       </c>
       <c r="D14" t="n">
-        <v>474.97</v>
+        <v>164.1</v>
       </c>
       <c r="E14" t="n">
-        <v>0.6</v>
+        <v>8.5</v>
       </c>
       <c r="F14" t="n">
-        <v>70.55</v>
+        <v>60.6</v>
       </c>
       <c r="G14" t="n">
-        <v>18.35</v>
+        <v>0.25</v>
       </c>
       <c r="H14" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>12-08-2026</t>
+          <t>24-06-2026</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SENCO</t>
+          <t>TRUALT</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>SENCO GOLD LIMITED</t>
+          <t>TRUALT BIOENERGY LIMITED</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>342</v>
+        <v>478</v>
       </c>
       <c r="D15" t="n">
-        <v>334.88</v>
+        <v>474.82</v>
       </c>
       <c r="E15" t="n">
-        <v>2.1</v>
+        <v>0.7</v>
       </c>
       <c r="F15" t="n">
-        <v>68.48</v>
+        <v>70.55</v>
       </c>
       <c r="G15" t="n">
-        <v>0.3</v>
+        <v>10.22</v>
       </c>
       <c r="H15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>30-06-2026</t>
+          <t>12-08-2026</t>
         </is>
       </c>
     </row>
@@ -4878,245 +4959,245 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>SENCO</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>HCL Technologies Limited</t>
+          <t>SENCO GOLD LIMITED</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1325</v>
+        <v>342</v>
       </c>
       <c r="D17" t="n">
-        <v>1104.34</v>
+        <v>334.88</v>
       </c>
       <c r="E17" t="n">
-        <v>20</v>
+        <v>2.1</v>
       </c>
       <c r="F17" t="n">
-        <v>60.82</v>
+        <v>68.48</v>
       </c>
       <c r="G17" t="n">
-        <v>5.22</v>
+        <v>0.3</v>
       </c>
       <c r="H17" t="n">
         <v>1</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>12-06-2026</t>
+          <t>30-06-2026</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>LAOPALA</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>LA OPALA RG LIMITED</t>
+          <t>HCL Technologies Limited</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>190.6</v>
+        <v>1325</v>
       </c>
       <c r="D18" t="n">
-        <v>173.91</v>
+        <v>1104.34</v>
       </c>
       <c r="E18" t="n">
-        <v>9.6</v>
+        <v>20</v>
       </c>
       <c r="F18" t="n">
-        <v>65.64</v>
+        <v>60.82</v>
       </c>
       <c r="G18" t="n">
-        <v>2.61</v>
+        <v>5.22</v>
       </c>
       <c r="H18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>08-06-2026</t>
+          <t>12-06-2026</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BAJAJHCARE</t>
+          <t>LAOPALA</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>BAJAJ HEALTHCARE LIMITED</t>
+          <t>LA OPALA RG LIMITED</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>323.05</v>
+        <v>190.6</v>
       </c>
       <c r="D19" t="n">
-        <v>297.3</v>
+        <v>173.91</v>
       </c>
       <c r="E19" t="n">
-        <v>8.699999999999999</v>
+        <v>9.6</v>
       </c>
       <c r="F19" t="n">
-        <v>67.69</v>
+        <v>65.64</v>
       </c>
       <c r="G19" t="n">
-        <v>2.97</v>
+        <v>2.61</v>
       </c>
       <c r="H19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>12-06-2026</t>
+          <t>08-06-2026</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MOTOGENFIN</t>
+          <t>BAJAJHCARE</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>THE MOTOR &amp; GENERAL FINANCE LIMITED</t>
+          <t>BAJAJ HEALTHCARE LIMITED</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>26.07</v>
+        <v>323.05</v>
       </c>
       <c r="D20" t="n">
-        <v>29.18</v>
+        <v>297.3</v>
       </c>
       <c r="E20" t="n">
-        <v>-10.7</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="F20" t="n">
-        <v>69.03</v>
+        <v>67.69</v>
       </c>
       <c r="G20" t="n">
-        <v>1.48</v>
+        <v>2.97</v>
       </c>
       <c r="H20" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>12-06-2026</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BMWVENTLTD</t>
+          <t>GANESHCP</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>BMW VENTURES LIMITED</t>
+          <t>GANESH CONSUMER PRODUCTS LIMITED</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>57.32</v>
+        <v>164.67</v>
       </c>
       <c r="D21" t="n">
-        <v>60.13</v>
+        <v>204.13</v>
       </c>
       <c r="E21" t="n">
-        <v>-4.7</v>
+        <v>-19.3</v>
       </c>
       <c r="F21" t="n">
-        <v>73.01000000000001</v>
+        <v>64.08</v>
       </c>
       <c r="G21" t="n">
-        <v>1.41</v>
+        <v>7.57</v>
       </c>
       <c r="H21" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>06-08-2026</t>
+          <t>30-06-2026</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>GANESHCP</t>
+          <t>ARSSBL</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>GANESH CONSUMER PRODUCTS LIMITED</t>
+          <t>Anand Rathi Share and Stock Brokers Limited</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>164.67</v>
+        <v>511.95</v>
       </c>
       <c r="D22" t="n">
-        <v>204.13</v>
+        <v>545.03</v>
       </c>
       <c r="E22" t="n">
-        <v>-19.3</v>
+        <v>-6.1</v>
       </c>
       <c r="F22" t="n">
-        <v>64.08</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="G22" t="n">
-        <v>7.57</v>
+        <v>1.09</v>
       </c>
       <c r="H22" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>30-06-2026</t>
+          <t>16-06-2026</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ARSSBL</t>
+          <t>AJMERA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Anand Rathi Share and Stock Brokers Limited</t>
+          <t>AJMERA REALTY &amp; INFRA INDIA LIMITED</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>511.95</v>
+        <v>119.6</v>
       </c>
       <c r="D23" t="n">
-        <v>545.03</v>
+        <v>114.86</v>
       </c>
       <c r="E23" t="n">
-        <v>-6.1</v>
+        <v>4.1</v>
       </c>
       <c r="F23" t="n">
-        <v>69.90000000000001</v>
+        <v>69.73999999999999</v>
       </c>
       <c r="G23" t="n">
-        <v>2.18</v>
+        <v>7.36</v>
       </c>
       <c r="H23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>16-06-2026</t>
+          <t>04-06-2026</t>
         </is>
       </c>
     </row>
@@ -5158,35 +5239,35 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AJMERA</t>
+          <t>MOTOGENFIN</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>AJMERA REALTY &amp; INFRA INDIA LIMITED</t>
+          <t>THE MOTOR &amp; GENERAL FINANCE LIMITED</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>119.6</v>
+        <v>26.07</v>
       </c>
       <c r="D25" t="n">
-        <v>114.86</v>
+        <v>29.14</v>
       </c>
       <c r="E25" t="n">
-        <v>4.1</v>
+        <v>-10.5</v>
       </c>
       <c r="F25" t="n">
-        <v>69.73999999999999</v>
+        <v>69.03</v>
       </c>
       <c r="G25" t="n">
-        <v>7.36</v>
+        <v>1.34</v>
       </c>
       <c r="H25" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>04-06-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
     </row>
@@ -5263,70 +5344,70 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>OMPOWER</t>
+          <t>THOMASCOOK</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Om Power Transmission Limited</t>
+          <t>THOMAS COOK (INDIA) LIMITED</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>167.95</v>
+        <v>103.75</v>
       </c>
       <c r="D28" t="n">
-        <v>182.69</v>
+        <v>109.31</v>
       </c>
       <c r="E28" t="n">
-        <v>-8.1</v>
+        <v>-5.1</v>
       </c>
       <c r="F28" t="n">
-        <v>69.05</v>
+        <v>72.34</v>
       </c>
       <c r="G28" t="n">
-        <v>0.74</v>
+        <v>48.4</v>
       </c>
       <c r="H28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>24-06-2026</t>
+          <t>11-06-2026</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>THOMASCOOK</t>
+          <t>OMPOWER</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>THOMAS COOK (INDIA) LIMITED</t>
+          <t>Om Power Transmission Limited</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>103.75</v>
+        <v>167.95</v>
       </c>
       <c r="D29" t="n">
-        <v>109.31</v>
+        <v>182.69</v>
       </c>
       <c r="E29" t="n">
-        <v>-5.1</v>
+        <v>-8.1</v>
       </c>
       <c r="F29" t="n">
-        <v>72.34</v>
+        <v>69.05</v>
       </c>
       <c r="G29" t="n">
-        <v>48.4</v>
+        <v>0.74</v>
       </c>
       <c r="H29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>11-06-2026</t>
+          <t>24-06-2026</t>
         </is>
       </c>
     </row>
@@ -5368,70 +5449,70 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>GRMOVER</t>
+          <t>BMWVENTLTD</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>GRM OVERSEAS LIMITED</t>
+          <t>BMW VENTURES LIMITED</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>90</v>
+        <v>57.32</v>
       </c>
       <c r="D31" t="n">
-        <v>100.13</v>
+        <v>60.15</v>
       </c>
       <c r="E31" t="n">
-        <v>-10.1</v>
+        <v>-4.7</v>
       </c>
       <c r="F31" t="n">
-        <v>71.72</v>
+        <v>73.01000000000001</v>
       </c>
       <c r="G31" t="n">
-        <v>15.9</v>
+        <v>0.9</v>
       </c>
       <c r="H31" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>24-06-2026</t>
+          <t>06-08-2026</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>MANINFRA</t>
+          <t>GRMOVER</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MAN INFRACONSTRUCTION LIMITED</t>
+          <t>GRM OVERSEAS LIMITED</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="D32" t="n">
-        <v>105.19</v>
+        <v>95.54000000000001</v>
       </c>
       <c r="E32" t="n">
-        <v>-1.1</v>
+        <v>-5.8</v>
       </c>
       <c r="F32" t="n">
-        <v>67.15000000000001</v>
+        <v>71.72</v>
       </c>
       <c r="G32" t="n">
-        <v>7.89</v>
+        <v>10.87</v>
       </c>
       <c r="H32" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>24-06-2026</t>
         </is>
       </c>
     </row>
@@ -5450,19 +5531,19 @@
         <v>74.34999999999999</v>
       </c>
       <c r="D33" t="n">
-        <v>74.84999999999999</v>
+        <v>74.92</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.7</v>
+        <v>-0.8</v>
       </c>
       <c r="F33" t="n">
         <v>62.78</v>
       </c>
       <c r="G33" t="n">
-        <v>1.8</v>
+        <v>1.48</v>
       </c>
       <c r="H33" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -5555,19 +5636,19 @@
         <v>285</v>
       </c>
       <c r="D36" t="n">
-        <v>297.22</v>
+        <v>292.28</v>
       </c>
       <c r="E36" t="n">
-        <v>-4.1</v>
+        <v>-2.5</v>
       </c>
       <c r="F36" t="n">
         <v>70.45</v>
       </c>
       <c r="G36" t="n">
-        <v>1.9</v>
+        <v>1.29</v>
       </c>
       <c r="H36" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
@@ -5578,103 +5659,138 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>VSTL</t>
+          <t>MANINFRA</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>VIBHOR STEEL TUBES LIMITED</t>
+          <t>MAN INFRACONSTRUCTION LIMITED</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>106.8</v>
+        <v>104</v>
       </c>
       <c r="D37" t="n">
-        <v>117.88</v>
+        <v>105.19</v>
       </c>
       <c r="E37" t="n">
-        <v>-9.4</v>
+        <v>-1.1</v>
       </c>
       <c r="F37" t="n">
-        <v>73.48</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="G37" t="n">
-        <v>0.27</v>
+        <v>2.63</v>
       </c>
       <c r="H37" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>12-06-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>WCIL</t>
+          <t>VSTL</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>WESTERN CARRIERS (INDIA) LIMITED</t>
+          <t>VIBHOR STEEL TUBES LIMITED</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>87.98</v>
+        <v>106.8</v>
       </c>
       <c r="D38" t="n">
-        <v>100.33</v>
+        <v>117.88</v>
       </c>
       <c r="E38" t="n">
-        <v>-12.3</v>
+        <v>-9.4</v>
       </c>
       <c r="F38" t="n">
-        <v>71.89</v>
+        <v>73.48</v>
       </c>
       <c r="G38" t="n">
-        <v>0.63</v>
+        <v>0.27</v>
       </c>
       <c r="H38" t="n">
         <v>5</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>30-06-2026</t>
+          <t>12-06-2026</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>WCIL</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>WESTERN CARRIERS (INDIA) LIMITED</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>87.98</v>
+      </c>
+      <c r="D39" t="n">
+        <v>100.33</v>
+      </c>
+      <c r="E39" t="n">
+        <v>-12.3</v>
+      </c>
+      <c r="F39" t="n">
+        <v>71.89</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="H39" t="n">
+        <v>5</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>30-06-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>TIGERLOGS</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>Tiger Logistics (India) Limited</t>
         </is>
       </c>
-      <c r="C39" t="n">
+      <c r="C40" t="n">
         <v>26.8</v>
       </c>
-      <c r="D39" t="n">
+      <c r="D40" t="n">
         <v>36.7</v>
       </c>
-      <c r="E39" t="n">
+      <c r="E40" t="n">
         <v>-27</v>
       </c>
-      <c r="F39" t="n">
+      <c r="F40" t="n">
         <v>61.81</v>
       </c>
-      <c r="G39" t="n">
+      <c r="G40" t="n">
         <v>0.66</v>
       </c>
-      <c r="H39" t="n">
+      <c r="H40" t="n">
         <v>10</v>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>30-06-2026</t>
         </is>
@@ -5695,12 +5811,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Band</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
@@ -5713,7 +5829,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3">
@@ -5723,7 +5839,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -5743,7 +5859,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
@@ -5773,7 +5889,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9">
@@ -5783,7 +5899,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
@@ -5803,7 +5919,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>